<commit_message>
Added new prompting strategy and new excel
</commit_message>
<xml_diff>
--- a/src/npr/demo_clean.xlsx
+++ b/src/npr/demo_clean.xlsx
@@ -413,31 +413,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Série avec les masques de DICOM SEG</t>
+          <t xml:space="preserve">Série avec les masques de DICOM SEG
+</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>lesion size in mm</t>
+          <t>PatientID</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>PatientID</t>
+          <t>AccessionNumber</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>AccessionNumber</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>Clinical information data (Pseudo reports)</t>
         </is>
@@ -451,25 +447,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>55.1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>0301B7D6</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="C2" t="n">
         <v>11092835</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>- Right upper parahilar central lung mass difficult to measure (NON-TARGET lesion) without significant changes, with signs of infiltration of mediastinal fat with infiltration of the SVC, compatible with unchanged primary pulmonary neoproliferative process.
 - Significant increase in size of the high right paratracheal mediastinal adenopathic involvement that is difficult to delimit.
-- F1  Right paravertebral apical pulmonary nodule of 20x14mm unchanged, neoplastic appearance (image 11), with associated fibroscarrial lesion apical right apical, without significant changes.
+- (F1) Right paravertebral apical pulmonary nodule of 55 mm unchanged, neoplastic appearance (Image-9), with associated fibroscarrial lesion apical right apical, without significant changes.
 - Pseudonodular condensation with a fibrocicatricial appearance in the left posterior costophrenic sinus unchanged, with the appearance of atelectatic condensation in the right posterior costophrenic sinus.
 - No evidence of other nodules or suspicious lung condensations.
-- No pleural effusion.</t>
+- No pleural effusion.
+- Left adrenal nodular lesion of 14 mm (anterior of 16 mm) (image 21) suspicious of M1.
+- Sclerosing changes in the trabecular bone of the body and the glen of the right scapula, with a lytic component in the region of the acromion compatible with metastatic lesion, probably related to radial changes according to CLINICAL INFORMATION.</t>
         </is>
       </c>
     </row>
@@ -481,24 +474,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">59.0
-37.4
-10.7
-17.3
-</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>0301B7D6</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="C3" t="n">
         <v>11297707</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>"Patient with PsA of Lung Neoplasia"</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>"Thoracic, abdominal, and pelvic CT scans are performed after administration of ev contrast."</t>
         </is>
       </c>
     </row>
@@ -510,23 +494,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>34.3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
           <t>0301B7D6</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="C4" t="n">
         <v>31981427</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Here is the extracted text containing only the pulmonary or thoracic findings:
-"right upper parahilar central lung mass that is difficult to measure (non-target lesion), with signs of infiltration of mediastinal fat with infiltration of the VCS, compatible with primary pulmonary neoproliferative process. High right paratracheal mediastinal adenopathic involvement difficult to delimit (non-target lesion).
-F1 A 20x27mm right paravertebral apical pulmonary nodule with a neoplastic appearance (image 15) with a fibrocitricial lesion associated with the right apical appearance. Pseudonodular condensation with fibrocicatricial appearance in the left posterior costophrenic sinus.
-There is no evidence of other nodules or suspicious pulmonary condensations. Do not have pleural effusion."</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>right upper parahilar central lung mass that is difficult to measure (non-target lesion), with signs of infiltration of mediastinal fat with infiltration of the VCS, compatible with primary pulmonary neoproliferative process.
+High right paratracheal mediastinal adenopathic involvement difficult to delimit (non-target lesion).
+(F1) A 32 mm right paravertebral apical pulmonary nodule with a neoplastic appearance (image -14) with a fibrocitricial lesion associated with the right apical appearance.
+Pseudonodular condensation with fibrocicatricial appearance in the left posterior costophrenic sinus.
+There is no evidence of other nodules or suspicious pulmonary condensations. Do not have pleural effusion.
+Left adrenal nodular lesion measuring 26x21mm, suspicious of M1.</t>
         </is>
       </c>
     </row>
@@ -538,25 +519,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>42.8</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
           <t>0301B7D6</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="C5" t="n">
         <v>57329381</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>- Right upper parahilar central lung mass difficult to measure (NON-TARGET lesion) without significant changes, with signs of infiltration of mediastinal fat with infiltration of the SVC, compatible with primary pulmonary neoproliferative process.
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>- Size stability of lymph nodes in the right supraclavicular fossa, among which we highlight the largest of 27x42 (anterior of 27x39mm)(image 3)
+- Right axillary lymphadenopathy of 13x15mm (anterior of 18x24mm)(image 21)
+- Right upper parahilar central lung mass difficult to measure (NON-TARGET lesion) without significant changes, with signs of infiltration of mediastinal fat with infiltration of the SVC, compatible with primary pulmonary neoproliferative process.
 - High right paratracheal mediastinal adenopathic involvement difficult to delimit (NON-TARGET lesion) without relevant changes.
-- F1 Right paravertebral apical pulmonary nodule of 25x22mm (anterior of 20x27mm), neoplastic appearance (image 10), with lesion of associated fibroscarrial appearance of right apical, without significant changes.
-- Pseudonodular condensation with fibroscarrial appearance in left posterior costophrenic sinus unchanged.
+-(F1) Right paravertebral apical pulmonary nodule of 43mm, neoplastic appearance (image 9), with lesion of associated fibroscarrial appearance of right apical, without significant changes.
 - No evidence of other nodules or suspicious lung condensations.
-- No pleural effusion.</t>
+- No pleural effusion.
+- Left adrenal nodular lesion of 25 mm (anterior of 26 mm) suspicious of M1.</t>
         </is>
       </c>
     </row>
@@ -568,25 +546,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>44.9</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>0301B7D6</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="C6" t="n">
         <v>92106962</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>- Right upper parahilar central lung mass difficult to measure (NON-TARGET lesion) without significant changes, with signs of infiltration of mediastinal fat with infiltration of the SVC, compatible with primary pulmonary neoproliferative process.
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>- Increase in the size of lymphadenopathies in the right supraclavicular fossa, among which we highlight the largest of 36x54 (anterior of 27x42mm)(image 4)
+- Right axillary lymphadenopathy of 13x15mm unchanged (image 25)
+- Right upper parahilar central lung mass difficult to measure (NON-TARGET lesion) without significant changes, with signs of infiltration of mediastinal fat with infiltration of the SVC, compatible with primary pulmonary neoproliferative process.
 - Significant increase in size of the high right paratracheal mediastinal adenopathic involvement that is difficult to delimit.
-- L1 Right paravertebral apical pulmonary nodule of 20x14mm (anterior of 25x22mm), neoplastic appearance (image 10), with a lesion of associated fibroscarrial appearance of right apical, without significant changes.
-- Pseudonodular condensation with fibroscarrial appearance in left posterior costophrenic sinus unchanged.
+- (F1) Right paravertebral apical pulmonary nodule of 44 mm, neoplastic appearance (image 12), with a lesion of associated fibroscarrial appearance of right apical, without significant changes.
+Pseudonodular condensation with fibroscarrial appearance in left posterior costophrenic sinus unchanged.
 - No evidence of other nodules or suspicious lung condensations.
-- No pleural effusion.</t>
+- No pleural effusion.
+- Left adrenal nodular lesion of 16 mm (anterior of 25 mm) (image 19) suspected of M1.</t>
         </is>
       </c>
     </row>

</xml_diff>